<commit_message>
Add total quantity (pcs) per HS code to Fired Up CZ26010445 summary
Insert a Quantity (pcs) column showing consolidated units per HS code
(total 8 426 pcs), alongside the existing gross weight and customs value.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01A1rgrnUnArwBCa31fbGGfH
</commit_message>
<xml_diff>
--- a/output/HS_Code_Summary_Fired_Up_CZ26010445.xlsx
+++ b/output/HS_Code_Summary_Fired_Up_CZ26010445.xlsx
@@ -119,7 +119,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -137,6 +137,9 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="4" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -146,6 +149,9 @@
     <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="3" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="4" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -153,6 +159,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="4" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -527,16 +536,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G38"/>
+  <dimension ref="A1:H38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
-    <col width="46" customWidth="1" min="2" max="2"/>
+    <col width="44" customWidth="1" min="2" max="2"/>
     <col width="26" customWidth="1" min="3" max="3"/>
-    <col width="15" customWidth="1" min="4" max="4"/>
-    <col width="17" customWidth="1" min="5" max="5"/>
-    <col width="9" customWidth="1" min="6" max="6"/>
-    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="17" customWidth="1" min="6" max="6"/>
+    <col width="9" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -584,20 +594,25 @@
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
+          <t>Quantity (pcs)</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
           <t>Gross weight (kg)</t>
         </is>
       </c>
-      <c r="E5" s="4" t="inlineStr">
+      <c r="F5" s="4" t="inlineStr">
         <is>
           <t>Customs value (GBP)</t>
         </is>
       </c>
-      <c r="F5" s="4" t="inlineStr">
+      <c r="G5" s="4" t="inlineStr">
         <is>
           <t>CBAM</t>
         </is>
       </c>
-      <c r="G5" s="4" t="inlineStr">
+      <c r="H5" s="4" t="inlineStr">
         <is>
           <t>Antidumping</t>
         </is>
@@ -620,17 +635,20 @@
         </is>
       </c>
       <c r="D6" s="7" t="n">
+        <v>1420</v>
+      </c>
+      <c r="E6" s="8" t="n">
         <v>297.19</v>
       </c>
-      <c r="E6" s="7" t="n">
+      <c r="F6" s="8" t="n">
         <v>1539.08</v>
       </c>
-      <c r="F6" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H6" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -653,17 +671,20 @@
         </is>
       </c>
       <c r="D7" s="7" t="n">
+        <v>216</v>
+      </c>
+      <c r="E7" s="8" t="n">
         <v>45.36</v>
       </c>
-      <c r="E7" s="7" t="n">
+      <c r="F7" s="8" t="n">
         <v>552.96</v>
       </c>
-      <c r="F7" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="G7" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H7" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -686,17 +707,20 @@
         </is>
       </c>
       <c r="D8" s="7" t="n">
+        <v>20</v>
+      </c>
+      <c r="E8" s="8" t="n">
         <v>52</v>
       </c>
-      <c r="E8" s="7" t="n">
+      <c r="F8" s="8" t="n">
         <v>206.6</v>
       </c>
-      <c r="F8" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="G8" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H8" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -719,83 +743,92 @@
         </is>
       </c>
       <c r="D9" s="7" t="n">
+        <v>60</v>
+      </c>
+      <c r="E9" s="8" t="n">
         <v>23.4</v>
       </c>
-      <c r="E9" s="7" t="n">
+      <c r="F9" s="8" t="n">
         <v>233.4</v>
       </c>
-      <c r="F9" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
+      <c r="H9" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" s="8" t="inlineStr">
+      <c r="A10" s="9" t="inlineStr">
         <is>
           <t>48030090</t>
         </is>
       </c>
-      <c r="B10" s="9" t="inlineStr">
+      <c r="B10" s="10" t="inlineStr">
         <is>
           <t>Kapesníčky (facial tissues)</t>
         </is>
       </c>
-      <c r="C10" s="8" t="inlineStr">
+      <c r="C10" s="9" t="inlineStr">
         <is>
           <t>GB (preferential UK origin)</t>
         </is>
       </c>
-      <c r="D10" s="10" t="n">
+      <c r="D10" s="11" t="n">
+        <v>2560</v>
+      </c>
+      <c r="E10" s="12" t="n">
         <v>401.92</v>
       </c>
-      <c r="E10" s="10" t="n">
+      <c r="F10" s="12" t="n">
         <v>921.6</v>
       </c>
-      <c r="F10" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G10" s="8" t="inlineStr">
+      <c r="G10" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H10" s="9" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="8" t="inlineStr">
+      <c r="A11" s="9" t="inlineStr">
         <is>
           <t>49111010</t>
         </is>
       </c>
-      <c r="B11" s="9" t="inlineStr">
+      <c r="B11" s="10" t="inlineStr">
         <is>
           <t>Brožury (brochures)</t>
         </is>
       </c>
-      <c r="C11" s="8" t="inlineStr">
+      <c r="C11" s="9" t="inlineStr">
         <is>
           <t>GB (preferential UK origin)</t>
         </is>
       </c>
-      <c r="D11" s="10" t="n">
+      <c r="D11" s="11" t="n">
+        <v>5</v>
+      </c>
+      <c r="E11" s="12" t="n">
         <v>63</v>
       </c>
-      <c r="E11" s="10" t="n">
+      <c r="F11" s="12" t="n">
         <v>0.5</v>
       </c>
-      <c r="F11" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G11" s="8" t="inlineStr">
+      <c r="G11" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H11" s="9" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -818,17 +851,20 @@
         </is>
       </c>
       <c r="D12" s="7" t="n">
+        <v>300</v>
+      </c>
+      <c r="E12" s="8" t="n">
         <v>18</v>
       </c>
-      <c r="E12" s="7" t="n">
+      <c r="F12" s="8" t="n">
         <v>384</v>
       </c>
-      <c r="F12" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="G12" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H12" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -851,17 +887,20 @@
         </is>
       </c>
       <c r="D13" s="7" t="n">
+        <v>120</v>
+      </c>
+      <c r="E13" s="8" t="n">
         <v>136.8</v>
       </c>
-      <c r="E13" s="7" t="n">
+      <c r="F13" s="8" t="n">
         <v>1303.2</v>
       </c>
-      <c r="F13" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="G13" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H13" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -884,17 +923,20 @@
         </is>
       </c>
       <c r="D14" s="7" t="n">
+        <v>35</v>
+      </c>
+      <c r="E14" s="8" t="n">
         <v>829.7</v>
       </c>
-      <c r="E14" s="7" t="n">
+      <c r="F14" s="8" t="n">
         <v>3612.1</v>
       </c>
-      <c r="F14" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="G14" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H14" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -917,17 +959,20 @@
         </is>
       </c>
       <c r="D15" s="7" t="n">
+        <v>200</v>
+      </c>
+      <c r="E15" s="8" t="n">
         <v>57</v>
       </c>
-      <c r="E15" s="7" t="n">
+      <c r="F15" s="8" t="n">
         <v>860</v>
       </c>
-      <c r="F15" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="G15" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H15" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -950,17 +995,20 @@
         </is>
       </c>
       <c r="D16" s="7" t="n">
+        <v>540</v>
+      </c>
+      <c r="E16" s="8" t="n">
         <v>144</v>
       </c>
-      <c r="E16" s="7" t="n">
+      <c r="F16" s="8" t="n">
         <v>913.2</v>
       </c>
-      <c r="F16" s="11" t="inlineStr">
+      <c r="G16" s="13" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="G16" s="5" t="inlineStr">
+      <c r="H16" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -983,17 +1031,20 @@
         </is>
       </c>
       <c r="D17" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="E17" s="8" t="n">
         <v>33</v>
       </c>
-      <c r="E17" s="7" t="n">
+      <c r="F17" s="8" t="n">
         <v>10</v>
       </c>
-      <c r="F17" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="G17" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H17" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1016,17 +1067,20 @@
         </is>
       </c>
       <c r="D18" s="7" t="n">
+        <v>50</v>
+      </c>
+      <c r="E18" s="8" t="n">
         <v>570.3</v>
       </c>
-      <c r="E18" s="7" t="n">
+      <c r="F18" s="8" t="n">
         <v>1972.5</v>
       </c>
-      <c r="F18" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="G18" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H18" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1049,17 +1103,20 @@
         </is>
       </c>
       <c r="D19" s="7" t="n">
+        <v>93</v>
+      </c>
+      <c r="E19" s="8" t="n">
         <v>1171.8</v>
       </c>
-      <c r="E19" s="7" t="n">
+      <c r="F19" s="8" t="n">
         <v>5477.07</v>
       </c>
-      <c r="F19" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="G19" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H19" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1082,50 +1139,56 @@
         </is>
       </c>
       <c r="D20" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="E20" s="8" t="n">
         <v>180</v>
       </c>
-      <c r="E20" s="7" t="n">
+      <c r="F20" s="8" t="n">
         <v>712</v>
       </c>
-      <c r="F20" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="G20" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
+      <c r="H20" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="21">
-      <c r="A21" s="8" t="inlineStr">
+      <c r="A21" s="9" t="inlineStr">
         <is>
           <t>84513000</t>
         </is>
       </c>
-      <c r="B21" s="9" t="inlineStr">
+      <c r="B21" s="10" t="inlineStr">
         <is>
           <t>Napařovačka/pukovačka na kalhoty (trouser press)</t>
         </is>
       </c>
-      <c r="C21" s="8" t="inlineStr">
+      <c r="C21" s="9" t="inlineStr">
         <is>
           <t>GB (preferential UK origin)</t>
         </is>
       </c>
-      <c r="D21" s="10" t="n">
+      <c r="D21" s="11" t="n">
+        <v>100</v>
+      </c>
+      <c r="E21" s="12" t="n">
         <v>1108.15</v>
       </c>
-      <c r="E21" s="10" t="n">
+      <c r="F21" s="12" t="n">
         <v>5211.55</v>
       </c>
-      <c r="F21" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G21" s="8" t="inlineStr">
+      <c r="G21" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H21" s="9" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1148,50 +1211,56 @@
         </is>
       </c>
       <c r="D22" s="7" t="n">
+        <v>2005</v>
+      </c>
+      <c r="E22" s="8" t="n">
         <v>172.5</v>
       </c>
-      <c r="E22" s="7" t="n">
+      <c r="F22" s="8" t="n">
         <v>621.5</v>
       </c>
-      <c r="F22" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="G22" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
+      <c r="H22" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="23">
-      <c r="A23" s="8" t="inlineStr">
+      <c r="A23" s="9" t="inlineStr">
         <is>
           <t>85162991</t>
         </is>
       </c>
-      <c r="B23" s="9" t="inlineStr">
+      <c r="B23" s="10" t="inlineStr">
         <is>
           <t>Elektrický nástěnný krb (wall fire)</t>
         </is>
       </c>
-      <c r="C23" s="8" t="inlineStr">
+      <c r="C23" s="9" t="inlineStr">
         <is>
           <t>GB (preferential UK origin)</t>
         </is>
       </c>
-      <c r="D23" s="10" t="n">
+      <c r="D23" s="11" t="n">
+        <v>15</v>
+      </c>
+      <c r="E23" s="12" t="n">
         <v>346.5</v>
       </c>
-      <c r="E23" s="10" t="n">
+      <c r="F23" s="12" t="n">
         <v>1232.7</v>
       </c>
-      <c r="F23" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G23" s="8" t="inlineStr">
+      <c r="G23" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H23" s="9" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1214,17 +1283,20 @@
         </is>
       </c>
       <c r="D24" s="7" t="n">
+        <v>189</v>
+      </c>
+      <c r="E24" s="8" t="n">
         <v>142.41</v>
       </c>
-      <c r="E24" s="7" t="n">
+      <c r="F24" s="8" t="n">
         <v>762.25</v>
       </c>
-      <c r="F24" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="G24" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H24" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1247,17 +1319,20 @@
         </is>
       </c>
       <c r="D25" s="7" t="n">
+        <v>120</v>
+      </c>
+      <c r="E25" s="8" t="n">
         <v>99.59999999999999</v>
       </c>
-      <c r="E25" s="7" t="n">
+      <c r="F25" s="8" t="n">
         <v>868.8</v>
       </c>
-      <c r="F25" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="G25" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H25" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1280,17 +1355,20 @@
         </is>
       </c>
       <c r="D26" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="E26" s="8" t="n">
         <v>69.69</v>
       </c>
-      <c r="E26" s="7" t="n">
+      <c r="F26" s="8" t="n">
         <v>906.5</v>
       </c>
-      <c r="F26" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="G26" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H26" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1313,17 +1391,20 @@
         </is>
       </c>
       <c r="D27" s="7" t="n">
+        <v>18</v>
+      </c>
+      <c r="E27" s="8" t="n">
         <v>51.84</v>
       </c>
-      <c r="E27" s="7" t="n">
+      <c r="F27" s="8" t="n">
         <v>470.34</v>
       </c>
-      <c r="F27" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="G27" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H27" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1346,94 +1427,100 @@
         </is>
       </c>
       <c r="D28" s="7" t="n">
+        <v>150</v>
+      </c>
+      <c r="E28" s="8" t="n">
         <v>666</v>
       </c>
-      <c r="E28" s="7" t="n">
+      <c r="F28" s="8" t="n">
         <v>2875.5</v>
       </c>
-      <c r="F28" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="G28" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
+      <c r="H28" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="29">
-      <c r="A29" s="12" t="inlineStr">
+      <c r="A29" s="14" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B29" s="12" t="n"/>
-      <c r="C29" s="12" t="inlineStr">
+      <c r="B29" s="14" t="n"/>
+      <c r="C29" s="14" t="inlineStr">
         <is>
           <t>22 HS codes</t>
         </is>
       </c>
-      <c r="D29" s="13" t="n">
+      <c r="D29" s="15" t="n">
+        <v>8426</v>
+      </c>
+      <c r="E29" s="16" t="n">
         <v>6680.16</v>
       </c>
-      <c r="E29" s="13" t="n">
+      <c r="F29" s="16" t="n">
         <v>31647.35</v>
       </c>
-      <c r="F29" s="12" t="n"/>
-      <c r="G29" s="12" t="n"/>
+      <c r="G29" s="14" t="n"/>
+      <c r="H29" s="14" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="14" t="inlineStr">
+      <c r="A31" s="17" t="inlineStr">
         <is>
           <t>Notes / compliance</t>
         </is>
       </c>
     </row>
     <row r="32" ht="30" customHeight="1">
-      <c r="A32" s="15" t="inlineStr">
+      <c r="A32" s="18" t="inlineStr">
         <is>
           <t>• Consolidation: line items merged to unique HS codes. HS 8516 29 91 is split by origin (GB vs CN) because origin changes the duty rate — GB rows are preferential, CN rows are not.</t>
         </is>
       </c>
     </row>
     <row r="33" ht="30" customHeight="1">
-      <c r="A33" s="15" t="inlineStr">
+      <c r="A33" s="18" t="inlineStr">
         <is>
           <t>• Discount: no trade discount shown on the commercial invoice, so customs values equal invoice line values (no proportional discount applied).</t>
         </is>
       </c>
     </row>
     <row r="34" ht="30" customHeight="1">
-      <c r="A34" s="15" t="inlineStr">
+      <c r="A34" s="18" t="inlineStr">
         <is>
           <t>• CBAM: HS 7326 90 98 (ironing-board holders) falls within CBAM Annex I (iron &amp; steel). CBAM quarterly reporting applies. Other iron/steel codes present (7321, 7324) are outside CBAM's current commodity scope.</t>
         </is>
       </c>
     </row>
     <row r="35" ht="30" customHeight="1">
-      <c r="A35" s="15" t="inlineStr">
+      <c r="A35" s="18" t="inlineStr">
         <is>
           <t>• Russia sanctions (iron &amp; steel): invoice carries the required declaration that iron &amp; steel products (Reg. 833/2014, Annex XVII) contain no Russian-origin inputs — keep with the file; needed for the iron/steel items (7321, 7324, 7326).</t>
         </is>
       </c>
     </row>
     <row r="36" ht="30" customHeight="1">
-      <c r="A36" s="15" t="inlineStr">
+      <c r="A36" s="18" t="inlineStr">
         <is>
           <t>• Antidumping: no line item appears to be subject to an EU anti-dumping measure based on HS code + origin. Recommend a final TARIC check per commodity code at clearance to confirm.</t>
         </is>
       </c>
     </row>
     <row r="37" ht="30" customHeight="1">
-      <c r="A37" s="15" t="inlineStr">
+      <c r="A37" s="18" t="inlineStr">
         <is>
           <t>• Weights: gross weights are per-item from the packing list and sum to 6 680.16 kg. The documents declare a total gross of 7 214.15 kg — the ~534 kg difference is pallet tare (26 pallets), not allocated to individual HS codes.</t>
         </is>
       </c>
     </row>
     <row r="38" ht="30" customHeight="1">
-      <c r="A38" s="15" t="inlineStr">
+      <c r="A38" s="18" t="inlineStr">
         <is>
           <t>• Value note: invoice line values sum to 31 647.35 GBP (Ex VAT) as declared. Values are in GBP — convert to CZK at the customs rate on the day of clearance.</t>
         </is>
@@ -1441,17 +1528,17 @@
     </row>
   </sheetData>
   <mergeCells count="11">
-    <mergeCell ref="A32:G32"/>
-    <mergeCell ref="A36:G36"/>
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A31:G31"/>
-    <mergeCell ref="A3:G3"/>
-    <mergeCell ref="A34:G34"/>
-    <mergeCell ref="A35:G35"/>
-    <mergeCell ref="A38:G38"/>
-    <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A33:G33"/>
-    <mergeCell ref="A37:G37"/>
+    <mergeCell ref="A3:H3"/>
+    <mergeCell ref="A35:H35"/>
+    <mergeCell ref="A38:H38"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A33:H33"/>
+    <mergeCell ref="A36:H36"/>
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A37:H37"/>
+    <mergeCell ref="A32:H32"/>
+    <mergeCell ref="A31:H31"/>
+    <mergeCell ref="A34:H34"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add net weight per HS code to Fired Up CZ26010445 summary
Add a Net weight (kg) column alongside gross weight, taken per item from
the packing list. Net totals 5 850.03 kg, matching the documents.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01A1rgrnUnArwBCa31fbGGfH
</commit_message>
<xml_diff>
--- a/output/HS_Code_Summary_Fired_Up_CZ26010445.xlsx
+++ b/output/HS_Code_Summary_Fired_Up_CZ26010445.xlsx
@@ -536,17 +536,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H38"/>
+  <dimension ref="A1:I38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
-    <col width="44" customWidth="1" min="2" max="2"/>
-    <col width="26" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="15" customWidth="1" min="5" max="5"/>
-    <col width="17" customWidth="1" min="6" max="6"/>
-    <col width="9" customWidth="1" min="7" max="7"/>
-    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="25" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="9" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -604,15 +605,20 @@
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
+          <t>Net weight (kg)</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
           <t>Customs value (GBP)</t>
         </is>
       </c>
-      <c r="G5" s="4" t="inlineStr">
+      <c r="H5" s="4" t="inlineStr">
         <is>
           <t>CBAM</t>
         </is>
       </c>
-      <c r="H5" s="4" t="inlineStr">
+      <c r="I5" s="4" t="inlineStr">
         <is>
           <t>Antidumping</t>
         </is>
@@ -641,14 +647,17 @@
         <v>297.19</v>
       </c>
       <c r="F6" s="8" t="n">
+        <v>283.31</v>
+      </c>
+      <c r="G6" s="8" t="n">
         <v>1539.08</v>
       </c>
-      <c r="G6" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I6" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -677,14 +686,17 @@
         <v>45.36</v>
       </c>
       <c r="F7" s="8" t="n">
+        <v>44.28</v>
+      </c>
+      <c r="G7" s="8" t="n">
         <v>552.96</v>
       </c>
-      <c r="G7" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="H7" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I7" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -713,14 +725,17 @@
         <v>52</v>
       </c>
       <c r="F8" s="8" t="n">
+        <v>52</v>
+      </c>
+      <c r="G8" s="8" t="n">
         <v>206.6</v>
       </c>
-      <c r="G8" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="H8" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I8" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -749,14 +764,17 @@
         <v>23.4</v>
       </c>
       <c r="F9" s="8" t="n">
+        <v>20.04</v>
+      </c>
+      <c r="G9" s="8" t="n">
         <v>233.4</v>
       </c>
-      <c r="G9" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="H9" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I9" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -785,14 +803,17 @@
         <v>401.92</v>
       </c>
       <c r="F10" s="12" t="n">
+        <v>401.92</v>
+      </c>
+      <c r="G10" s="12" t="n">
         <v>921.6</v>
       </c>
-      <c r="G10" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="H10" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I10" s="9" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -821,14 +842,17 @@
         <v>63</v>
       </c>
       <c r="F11" s="12" t="n">
+        <v>63</v>
+      </c>
+      <c r="G11" s="12" t="n">
         <v>0.5</v>
       </c>
-      <c r="G11" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="H11" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I11" s="9" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -857,14 +881,17 @@
         <v>18</v>
       </c>
       <c r="F12" s="8" t="n">
+        <v>18</v>
+      </c>
+      <c r="G12" s="8" t="n">
         <v>384</v>
       </c>
-      <c r="G12" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="H12" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I12" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -893,14 +920,17 @@
         <v>136.8</v>
       </c>
       <c r="F13" s="8" t="n">
+        <v>112.8</v>
+      </c>
+      <c r="G13" s="8" t="n">
         <v>1303.2</v>
       </c>
-      <c r="G13" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="H13" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I13" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -929,14 +959,17 @@
         <v>829.7</v>
       </c>
       <c r="F14" s="8" t="n">
+        <v>689.34</v>
+      </c>
+      <c r="G14" s="8" t="n">
         <v>3612.1</v>
       </c>
-      <c r="G14" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="H14" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I14" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -965,14 +998,17 @@
         <v>57</v>
       </c>
       <c r="F15" s="8" t="n">
+        <v>43.6</v>
+      </c>
+      <c r="G15" s="8" t="n">
         <v>860</v>
       </c>
-      <c r="G15" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="H15" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I15" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1001,14 +1037,17 @@
         <v>144</v>
       </c>
       <c r="F16" s="8" t="n">
+        <v>122.7</v>
+      </c>
+      <c r="G16" s="8" t="n">
         <v>913.2</v>
       </c>
-      <c r="G16" s="13" t="inlineStr">
+      <c r="H16" s="13" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="H16" s="5" t="inlineStr">
+      <c r="I16" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1037,14 +1076,17 @@
         <v>33</v>
       </c>
       <c r="F17" s="8" t="n">
+        <v>32</v>
+      </c>
+      <c r="G17" s="8" t="n">
         <v>10</v>
       </c>
-      <c r="G17" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="H17" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I17" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1073,14 +1115,17 @@
         <v>570.3</v>
       </c>
       <c r="F18" s="8" t="n">
+        <v>525.2</v>
+      </c>
+      <c r="G18" s="8" t="n">
         <v>1972.5</v>
       </c>
-      <c r="G18" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="H18" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I18" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1109,14 +1154,17 @@
         <v>1171.8</v>
       </c>
       <c r="F19" s="8" t="n">
+        <v>1060.2</v>
+      </c>
+      <c r="G19" s="8" t="n">
         <v>5477.07</v>
       </c>
-      <c r="G19" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="H19" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I19" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1145,14 +1193,17 @@
         <v>180</v>
       </c>
       <c r="F20" s="8" t="n">
+        <v>150</v>
+      </c>
+      <c r="G20" s="8" t="n">
         <v>712</v>
       </c>
-      <c r="G20" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="H20" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I20" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1181,14 +1232,17 @@
         <v>1108.15</v>
       </c>
       <c r="F21" s="12" t="n">
+        <v>960.6</v>
+      </c>
+      <c r="G21" s="12" t="n">
         <v>5211.55</v>
       </c>
-      <c r="G21" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="H21" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I21" s="9" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1217,14 +1271,17 @@
         <v>172.5</v>
       </c>
       <c r="F22" s="8" t="n">
+        <v>165.75</v>
+      </c>
+      <c r="G22" s="8" t="n">
         <v>621.5</v>
       </c>
-      <c r="G22" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="H22" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I22" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1253,14 +1310,17 @@
         <v>346.5</v>
       </c>
       <c r="F23" s="12" t="n">
+        <v>277.5</v>
+      </c>
+      <c r="G23" s="12" t="n">
         <v>1232.7</v>
       </c>
-      <c r="G23" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="H23" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I23" s="9" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1289,14 +1349,17 @@
         <v>142.41</v>
       </c>
       <c r="F24" s="8" t="n">
+        <v>115.81</v>
+      </c>
+      <c r="G24" s="8" t="n">
         <v>762.25</v>
       </c>
-      <c r="G24" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="H24" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I24" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1325,14 +1388,17 @@
         <v>99.59999999999999</v>
       </c>
       <c r="F25" s="8" t="n">
+        <v>90</v>
+      </c>
+      <c r="G25" s="8" t="n">
         <v>868.8</v>
       </c>
-      <c r="G25" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="H25" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I25" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1361,14 +1427,17 @@
         <v>69.69</v>
       </c>
       <c r="F26" s="8" t="n">
+        <v>58.3</v>
+      </c>
+      <c r="G26" s="8" t="n">
         <v>906.5</v>
       </c>
-      <c r="G26" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="H26" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I26" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1397,14 +1466,17 @@
         <v>51.84</v>
       </c>
       <c r="F27" s="8" t="n">
+        <v>40.18</v>
+      </c>
+      <c r="G27" s="8" t="n">
         <v>470.34</v>
       </c>
-      <c r="G27" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="H27" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I27" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1433,14 +1505,17 @@
         <v>666</v>
       </c>
       <c r="F28" s="8" t="n">
+        <v>523.5</v>
+      </c>
+      <c r="G28" s="8" t="n">
         <v>2875.5</v>
       </c>
-      <c r="G28" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="H28" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I28" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1465,10 +1540,13 @@
         <v>6680.16</v>
       </c>
       <c r="F29" s="16" t="n">
+        <v>5850.03</v>
+      </c>
+      <c r="G29" s="16" t="n">
         <v>31647.35</v>
       </c>
-      <c r="G29" s="14" t="n"/>
       <c r="H29" s="14" t="n"/>
+      <c r="I29" s="14" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="17" t="inlineStr">
@@ -1515,7 +1593,7 @@
     <row r="37" ht="30" customHeight="1">
       <c r="A37" s="18" t="inlineStr">
         <is>
-          <t>• Weights: gross weights are per-item from the packing list and sum to 6 680.16 kg. The documents declare a total gross of 7 214.15 kg — the ~534 kg difference is pallet tare (26 pallets), not allocated to individual HS codes.</t>
+          <t>• Weights: gross and net weights are per-item from the packing list. Net sums to 5 850.03 kg (matches the docs). Line gross sums to 6 680.16 kg; the documents declare 7 214.15 kg total gross — the ~534 kg difference is pallet tare (26 pallets), not allocated to individual HS codes.</t>
         </is>
       </c>
     </row>
@@ -1528,17 +1606,17 @@
     </row>
   </sheetData>
   <mergeCells count="11">
-    <mergeCell ref="A3:H3"/>
-    <mergeCell ref="A35:H35"/>
-    <mergeCell ref="A38:H38"/>
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A33:H33"/>
-    <mergeCell ref="A36:H36"/>
-    <mergeCell ref="A1:H1"/>
-    <mergeCell ref="A37:H37"/>
-    <mergeCell ref="A32:H32"/>
-    <mergeCell ref="A31:H31"/>
-    <mergeCell ref="A34:H34"/>
+    <mergeCell ref="A2:I2"/>
+    <mergeCell ref="A33:I33"/>
+    <mergeCell ref="A37:I37"/>
+    <mergeCell ref="A32:I32"/>
+    <mergeCell ref="A36:I36"/>
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A31:I31"/>
+    <mergeCell ref="A3:I3"/>
+    <mergeCell ref="A34:I34"/>
+    <mergeCell ref="A35:I35"/>
+    <mergeCell ref="A38:I38"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Reconcile gross weight to declared PL total (7214.15 kg)
The packing list line items sum to 6 680.16 kg gross, but the declared
total gross is 7 214.15 kg; the 533.99 kg gap is pallet tare (26 pallets)
not broken down per line. Distribute that tare across HS codes in
proportion to gross so the Gross weight column ties to the declared
7 214.15 kg. Net weight (5 850.03 kg) already reconciles and is unchanged.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01A1rgrnUnArwBCa31fbGGfH
</commit_message>
<xml_diff>
--- a/output/HS_Code_Summary_Fired_Up_CZ26010445.xlsx
+++ b/output/HS_Code_Summary_Fired_Up_CZ26010445.xlsx
@@ -644,7 +644,7 @@
         <v>1420</v>
       </c>
       <c r="E6" s="8" t="n">
-        <v>297.19</v>
+        <v>320.95</v>
       </c>
       <c r="F6" s="8" t="n">
         <v>283.31</v>
@@ -683,7 +683,7 @@
         <v>216</v>
       </c>
       <c r="E7" s="8" t="n">
-        <v>45.36</v>
+        <v>48.99</v>
       </c>
       <c r="F7" s="8" t="n">
         <v>44.28</v>
@@ -722,7 +722,7 @@
         <v>20</v>
       </c>
       <c r="E8" s="8" t="n">
-        <v>52</v>
+        <v>56.16</v>
       </c>
       <c r="F8" s="8" t="n">
         <v>52</v>
@@ -761,7 +761,7 @@
         <v>60</v>
       </c>
       <c r="E9" s="8" t="n">
-        <v>23.4</v>
+        <v>25.27</v>
       </c>
       <c r="F9" s="8" t="n">
         <v>20.04</v>
@@ -800,7 +800,7 @@
         <v>2560</v>
       </c>
       <c r="E10" s="12" t="n">
-        <v>401.92</v>
+        <v>434.05</v>
       </c>
       <c r="F10" s="12" t="n">
         <v>401.92</v>
@@ -839,7 +839,7 @@
         <v>5</v>
       </c>
       <c r="E11" s="12" t="n">
-        <v>63</v>
+        <v>68.04000000000001</v>
       </c>
       <c r="F11" s="12" t="n">
         <v>63</v>
@@ -878,7 +878,7 @@
         <v>300</v>
       </c>
       <c r="E12" s="8" t="n">
-        <v>18</v>
+        <v>19.44</v>
       </c>
       <c r="F12" s="8" t="n">
         <v>18</v>
@@ -917,7 +917,7 @@
         <v>120</v>
       </c>
       <c r="E13" s="8" t="n">
-        <v>136.8</v>
+        <v>147.74</v>
       </c>
       <c r="F13" s="8" t="n">
         <v>112.8</v>
@@ -956,7 +956,7 @@
         <v>35</v>
       </c>
       <c r="E14" s="8" t="n">
-        <v>829.7</v>
+        <v>896.02</v>
       </c>
       <c r="F14" s="8" t="n">
         <v>689.34</v>
@@ -995,7 +995,7 @@
         <v>200</v>
       </c>
       <c r="E15" s="8" t="n">
-        <v>57</v>
+        <v>61.56</v>
       </c>
       <c r="F15" s="8" t="n">
         <v>43.6</v>
@@ -1034,7 +1034,7 @@
         <v>540</v>
       </c>
       <c r="E16" s="8" t="n">
-        <v>144</v>
+        <v>155.51</v>
       </c>
       <c r="F16" s="8" t="n">
         <v>122.7</v>
@@ -1073,7 +1073,7 @@
         <v>100</v>
       </c>
       <c r="E17" s="8" t="n">
-        <v>33</v>
+        <v>35.64</v>
       </c>
       <c r="F17" s="8" t="n">
         <v>32</v>
@@ -1112,7 +1112,7 @@
         <v>50</v>
       </c>
       <c r="E18" s="8" t="n">
-        <v>570.3</v>
+        <v>615.89</v>
       </c>
       <c r="F18" s="8" t="n">
         <v>525.2</v>
@@ -1151,7 +1151,7 @@
         <v>93</v>
       </c>
       <c r="E19" s="8" t="n">
-        <v>1171.8</v>
+        <v>1265.45</v>
       </c>
       <c r="F19" s="8" t="n">
         <v>1060.2</v>
@@ -1190,7 +1190,7 @@
         <v>100</v>
       </c>
       <c r="E20" s="8" t="n">
-        <v>180</v>
+        <v>194.39</v>
       </c>
       <c r="F20" s="8" t="n">
         <v>150</v>
@@ -1229,7 +1229,7 @@
         <v>100</v>
       </c>
       <c r="E21" s="12" t="n">
-        <v>1108.15</v>
+        <v>1196.73</v>
       </c>
       <c r="F21" s="12" t="n">
         <v>960.6</v>
@@ -1268,7 +1268,7 @@
         <v>2005</v>
       </c>
       <c r="E22" s="8" t="n">
-        <v>172.5</v>
+        <v>186.29</v>
       </c>
       <c r="F22" s="8" t="n">
         <v>165.75</v>
@@ -1307,7 +1307,7 @@
         <v>15</v>
       </c>
       <c r="E23" s="12" t="n">
-        <v>346.5</v>
+        <v>374.2</v>
       </c>
       <c r="F23" s="12" t="n">
         <v>277.5</v>
@@ -1346,7 +1346,7 @@
         <v>189</v>
       </c>
       <c r="E24" s="8" t="n">
-        <v>142.41</v>
+        <v>153.79</v>
       </c>
       <c r="F24" s="8" t="n">
         <v>115.81</v>
@@ -1385,7 +1385,7 @@
         <v>120</v>
       </c>
       <c r="E25" s="8" t="n">
-        <v>99.59999999999999</v>
+        <v>107.56</v>
       </c>
       <c r="F25" s="8" t="n">
         <v>90</v>
@@ -1424,7 +1424,7 @@
         <v>10</v>
       </c>
       <c r="E26" s="8" t="n">
-        <v>69.69</v>
+        <v>75.26000000000001</v>
       </c>
       <c r="F26" s="8" t="n">
         <v>58.3</v>
@@ -1463,7 +1463,7 @@
         <v>18</v>
       </c>
       <c r="E27" s="8" t="n">
-        <v>51.84</v>
+        <v>55.98</v>
       </c>
       <c r="F27" s="8" t="n">
         <v>40.18</v>
@@ -1502,7 +1502,7 @@
         <v>150</v>
       </c>
       <c r="E28" s="8" t="n">
-        <v>666</v>
+        <v>719.24</v>
       </c>
       <c r="F28" s="8" t="n">
         <v>523.5</v>
@@ -1537,7 +1537,7 @@
         <v>8426</v>
       </c>
       <c r="E29" s="16" t="n">
-        <v>6680.16</v>
+        <v>7214.15</v>
       </c>
       <c r="F29" s="16" t="n">
         <v>5850.03</v>
@@ -1593,7 +1593,7 @@
     <row r="37" ht="30" customHeight="1">
       <c r="A37" s="18" t="inlineStr">
         <is>
-          <t>• Weights: gross and net weights are per-item from the packing list. Net sums to 5 850.03 kg (matches the docs). Line gross sums to 6 680.16 kg; the documents declare 7 214.15 kg total gross — the ~534 kg difference is pallet tare (26 pallets), not allocated to individual HS codes.</t>
+          <t>• Weights: net weights are per-item from the packing list and sum to 5 850.03 kg (matches the docs). The packing list's own line gross weights sum to only 6 680.16 kg, whereas the declared total gross is 7 214.15 kg — the 533.99 kg difference is pallet tare (26 pallets) that the PL does not break down per line. That pallet weight has been distributed across the HS codes in proportion to gross, so the Gross weight column totals to the declared 7 214.15 kg.</t>
         </is>
       </c>
     </row>

</xml_diff>